<commit_message>
Added new folder and updated project
</commit_message>
<xml_diff>
--- a/Test_case/labsqajobs.qaharboor Test case.xlsx
+++ b/Test_case/labsqajobs.qaharboor Test case.xlsx
@@ -98,26 +98,27 @@
     <r>
       <rPr>
         <rFont val="Calibri"/>
+        <color theme="1"/>
         <sz val="9.0"/>
       </rPr>
-      <t xml:space="preserve">1. Open browser
-2. Enter URL: </t>
+      <t>1. Open browser
+2. Enter URL: "</t>
     </r>
     <r>
       <rPr>
         <rFont val="Calibri"/>
-        <color rgb="FF1155CC"/>
+        <color rgb="FF000000"/>
         <sz val="9.0"/>
-        <u/>
       </rPr>
       <t>https://labsqajobs.qaharbor.com/</t>
     </r>
     <r>
       <rPr>
         <rFont val="Calibri"/>
+        <color theme="1"/>
         <sz val="9.0"/>
       </rPr>
-      <t xml:space="preserve">
+      <t>"
 3. Wait for homepage to load
 4. Click on Login button
 5. Verify login page is displayed
@@ -243,6 +244,7 @@
     <r>
       <rPr>
         <rFont val="Calibri"/>
+        <color theme="1"/>
         <sz val="9.0"/>
       </rPr>
       <t xml:space="preserve">1. Open browser
@@ -251,15 +253,15 @@
     <r>
       <rPr>
         <rFont val="Calibri"/>
-        <color rgb="FF1155CC"/>
+        <color rgb="FF000000"/>
         <sz val="9.0"/>
-        <u/>
       </rPr>
       <t>https://labsqajobs.qaharbor.com/</t>
     </r>
     <r>
       <rPr>
         <rFont val="Calibri"/>
+        <color theme="1"/>
         <sz val="9.0"/>
       </rPr>
       <t xml:space="preserve">
@@ -655,7 +657,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="14">
+  <fonts count="13">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -716,12 +718,6 @@
     <font>
       <sz val="9.0"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="9.0"/>
-      <color rgb="FF0000FF"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -849,19 +845,19 @@
     <xf borderId="3" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="3" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="3" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="3" fillId="6" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="3" fillId="6" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="3" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="3" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="3" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="3" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -879,7 +875,7 @@
     <xf borderId="3" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="3" fillId="6" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="3" fillId="6" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -6628,15 +6624,13 @@
   </dataValidations>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="B2"/>
-    <hyperlink r:id="rId2" ref="D11"/>
-    <hyperlink r:id="rId3" ref="D14"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="portrait"/>
-  <drawing r:id="rId4"/>
+  <drawing r:id="rId2"/>
   <tableParts count="1">
-    <tablePart r:id="rId6"/>
+    <tablePart r:id="rId4"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>